<commit_message>
Update daily revenue report
</commit_message>
<xml_diff>
--- a/reports/daily_revenue.xlsx
+++ b/reports/daily_revenue.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Performance" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Daily Performance" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sources &amp; Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Daily Performance'!$A$1:$M$53</definedName>
@@ -2756,13 +2756,13 @@
         <v>11525.74</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>6926.65003</v>
+        <v>7081.19002</v>
       </c>
       <c r="E53" s="3" t="n">
         <v>2339.34</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>1399.62</v>
+        <v>1399.66</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>140</v>
@@ -2771,10 +2771,10 @@
         <v>139.328</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>9265.990030000001</v>
+        <v>9420.53002</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>-1146.40003</v>
+        <v>-1300.94002</v>
       </c>
       <c r="K53" s="3" t="n">
         <v>30000</v>
@@ -2844,7 +2844,7 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>469804.30923</v>
+        <v>469958.84922</v>
       </c>
     </row>
     <row r="5">
@@ -2864,7 +2864,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>551783.56907</v>
+        <v>551938.10906</v>
       </c>
     </row>
     <row r="7">
@@ -2874,7 +2874,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>82585.38093</v>
+        <v>82430.84093999999</v>
       </c>
     </row>
     <row r="8">
@@ -2884,7 +2884,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>126869.64</v>
+        <v>126869.68</v>
       </c>
     </row>
     <row r="9">
@@ -2914,7 +2914,7 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>5.019087072368141</v>
+        <v>5.019085489929509</v>
       </c>
     </row>
     <row r="12">
@@ -2954,7 +2954,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.3695932645573097</v>
+        <v>0.369714840580106</v>
       </c>
     </row>
     <row r="16">
@@ -2974,7 +2974,7 @@
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>0.4340860367073076</v>
+        <v>0.4342076127301039</v>
       </c>
     </row>
     <row r="18">
@@ -2984,7 +2984,7 @@
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>0.06496960530790849</v>
+        <v>0.06484802928511217</v>
       </c>
     </row>
   </sheetData>
@@ -3025,7 +3025,7 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>2026-04-24T15:18:09-05:00</t>
+          <t>2026-04-24T15:45:19-05:00</t>
         </is>
       </c>
     </row>

</xml_diff>